<commit_message>
Pogo connector changed, deliverables and BOM generated
</commit_message>
<xml_diff>
--- a/Design Files/RECPT_POGO-JST/BOM/Client-BOM-RECPT_POGO-JST.xlsx
+++ b/Design Files/RECPT_POGO-JST/BOM/Client-BOM-RECPT_POGO-JST.xlsx
@@ -83,13 +83,13 @@
     <t>J1</t>
   </si>
   <si>
-    <t>POGO RECPT 5A 36V</t>
-  </si>
-  <si>
-    <t>MG0422-F-RA</t>
-  </si>
-  <si>
-    <t>Shenzhen Tiwei Technology co. LTD</t>
+    <t>POGO RECPT 48V 3A</t>
+  </si>
+  <si>
+    <t>HY41226288AM0618W</t>
+  </si>
+  <si>
+    <t>Shenzhen Weixunda Electronic  Technology Ltd.</t>
   </si>
 </sst>
 </file>
@@ -102,7 +102,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,13 +155,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -699,148 +692,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>